<commit_message>
content: refresh video/podcast inputs (drop old WC2026 batch, add new stories/previews); README
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/podcast/input/queue.xlsx
+++ b/podcast/input/queue.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="251">
   <si>
     <t>story</t>
   </si>
@@ -641,6 +641,132 @@
   </si>
   <si>
     <t>podcast/output/story79/story79.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story80.txt</t>
+  </si>
+  <si>
+    <t>podcast/input/deeplove/deeplove9.mp4; podcast/input/deeplove/deeplove6.mp4; podcast/input/deeplove/deeplove8.mp4; podcast/input/deeplove/deeplove10.mp4; podcast/input/deeplove/deeplove1.mp4; podcast/input/deeplove/deeplove3.mp4; podcast/input/deeplove/deeplove2.mp4; podcast/input/deeplove/deeplove4.mp4; podcast/input/deeplove/deeplove11.mp4; podcast/input/deeplove/deeplove5.mp4; podcast/input/deeplove/deeplove7.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story80/story80.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story81.txt</t>
+  </si>
+  <si>
+    <t>ronaldogoalnew</t>
+  </si>
+  <si>
+    <t>podcast/input/ronaldogoalnew/ronaldogoalnew2.mp4; podcast/input/ronaldogoalnew/ronaldogoalnew1.mp4; podcast/input/ronaldogoalnew/ronaldogoalnew3.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story81/story81.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story82.txt</t>
+  </si>
+  <si>
+    <t>podcast/input/life/life12.mp4; podcast/input/life/life11.mp4; podcast/input/life/life3.mp4; podcast/input/life/life6.mp4; podcast/input/life/life2.mp4; podcast/input/life/life13.mp4; podcast/input/life/life9.mp4; podcast/input/life/life1.mp4; podcast/input/life/life14.mp4; podcast/input/life/life8.mp4; podcast/input/life/life7.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story82/story82.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story83.txt</t>
+  </si>
+  <si>
+    <t>bluelock</t>
+  </si>
+  <si>
+    <t>podcast/input/bluelock/bluelock4.mp4; podcast/input/bluelock/bluelock2.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story83/story83.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story84.txt</t>
+  </si>
+  <si>
+    <t>podcast/input/japanstudent/japanstudent1.mp4; podcast/input/japanstudent/japanstudent2.mp4; podcast/input/japanstudent/japanstudent3.mp4; podcast/input/japanstudent/japanstudent6.mp4; podcast/input/japanstudent/japanstudent7.mp4; podcast/input/japanstudent/japanstudent5.mp4; podcast/input/japanstudent/japanstudent8.mp4; podcast/input/japanstudent/japanstudent4.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story84/story84.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story85.txt</t>
+  </si>
+  <si>
+    <t>podcast/input/aotdemo/aotpeak4.mp4; podcast/input/aotdemo/Video Project 18.mp4; podcast/input/aotdemo/aotdemo3.mp4; podcast/input/aotdemo/aotpeak1.mp4; podcast/input/aotdemo/aotdemo2.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story85/story85.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story86.txt</t>
+  </si>
+  <si>
+    <t>animedemo</t>
+  </si>
+  <si>
+    <t>podcast/input/animedemo/animedemo1.mp4; podcast/input/animedemo/animedemo2.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story86/story86.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story87.txt</t>
+  </si>
+  <si>
+    <t>podcast/input/aotdemo/aotpeak4.mp4; podcast/input/aotdemo/aotdemo2.mp4; podcast/input/aotdemo/aotpeak1.mp4; podcast/input/aotdemo/Video Project 18.mp4; podcast/input/aotdemo/aotdemo3.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story87/story87.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story88.txt</t>
+  </si>
+  <si>
+    <t>japanesenew</t>
+  </si>
+  <si>
+    <t>podcast/input/japanesenew/reelsvideo.io_1782655706212.mp4; podcast/input/japanesenew/reelsvideo.io_1782655766160.mp4; podcast/input/japanesenew/japanesenew2.mp4; podcast/input/japanesenew/japanesenew5.mp4; podcast/input/japanesenew/japanesenew1.mp4; podcast/input/japanesenew/japanesenew4.mp4; podcast/input/japanesenew/reelsvideo.io_1782655703723.mp4; podcast/input/japanesenew/reelsvideo.io_1782655788880.mp4; podcast/input/japanesenew/reelsvideo.io_1782655739472.mp4; podcast/input/japanesenew/japanesenew3.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story88/story88.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story90.txt</t>
+  </si>
+  <si>
+    <t>podcast/input/lifebeauty/lifebeauty1.mp4; podcast/input/lifebeauty/lifebeauty3.mp4; podcast/input/lifebeauty/lifebeauty7.mp4; podcast/input/lifebeauty/lifebeauty9.mp4; podcast/input/lifebeauty/lifebeauty4.mp4; podcast/input/lifebeauty/lifebeauty10.mp4; podcast/input/lifebeauty/lifebeauty5.mp4; podcast/input/lifebeauty/lifebeauty8.mp4; podcast/input/lifebeauty/lifebeauty2.mp4; podcast/input/lifebeauty/lifebeauty6.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story89/story89.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/ronaldo&amp;messi/messiargentina3.mp4; podcast/input/ronaldo&amp;messi/messilastdance1.mp4; podcast/input/ronaldo&amp;messi/ronaldotx5.mp4; podcast/input/ronaldo&amp;messi/ronaldotx1.mp4; podcast/input/ronaldo&amp;messi/ronaldotx2.mp4; podcast/input/ronaldo&amp;messi/ronaldotx16.mp4; podcast/input/ronaldo&amp;messi/messiargentina6.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story90/story90.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story91.txt</t>
+  </si>
+  <si>
+    <t>podcast/input/neymarlastdance/neymarlastdance2.mp4; podcast/input/neymarlastdance/neymarlastdance5.mp4; podcast/input/neymarlastdance/neymarlastdance1.mp4; podcast/input/neymarlastdance/neymarlastdance4.mp4; podcast/input/neymarlastdance/neymarlastdance3.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story91/story91.mp4</t>
+  </si>
+  <si>
+    <t>podcast/input/story/story92.txt</t>
+  </si>
+  <si>
+    <t>podcast/input/japanstudent/japanstudent4.mp4; podcast/input/japanstudent/japanstudent8.mp4; podcast/input/japanstudent/japanstudent5.mp4; podcast/input/japanstudent/japanstudent3.mp4; podcast/input/japanstudent/japanstudent2.mp4; podcast/input/japanstudent/japanstudent7.mp4; podcast/input/japanstudent/japanstudent6.mp4; podcast/input/japanstudent/japanstudent1.mp4</t>
+  </si>
+  <si>
+    <t>podcast/output/story92/story92.mp4</t>
   </si>
 </sst>
 </file>
@@ -988,11 +1114,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="27.33203125" customWidth="1"/>
     <col min="2" max="2" width="15.21875" customWidth="1"/>
+    <col min="3" max="3" width="255.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1993,6 +2120,227 @@
         <v>208</v>
       </c>
     </row>
+    <row r="62" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B62" t="s">
+        <v>200</v>
+      </c>
+      <c r="C62" t="s">
+        <v>210</v>
+      </c>
+      <c r="D62" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="63" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B63" t="s">
+        <v>213</v>
+      </c>
+      <c r="C63" t="s">
+        <v>214</v>
+      </c>
+      <c r="D63" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="64" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B64" t="s">
+        <v>163</v>
+      </c>
+      <c r="C64" t="s">
+        <v>217</v>
+      </c>
+      <c r="D64" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="65" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B65" t="s">
+        <v>220</v>
+      </c>
+      <c r="C65" t="s">
+        <v>221</v>
+      </c>
+      <c r="D65" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="66" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B66" t="s">
+        <v>153</v>
+      </c>
+      <c r="C66" t="s">
+        <v>224</v>
+      </c>
+      <c r="D66" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="67" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B67" t="s">
+        <v>104</v>
+      </c>
+      <c r="C67" t="s">
+        <v>227</v>
+      </c>
+      <c r="D67" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="68" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B68" t="s">
+        <v>230</v>
+      </c>
+      <c r="C68" t="s">
+        <v>231</v>
+      </c>
+      <c r="D68" t="s">
+        <v>8</v>
+      </c>
+      <c r="E68" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="69" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B69" t="s">
+        <v>104</v>
+      </c>
+      <c r="C69" t="s">
+        <v>234</v>
+      </c>
+      <c r="D69" t="s">
+        <v>8</v>
+      </c>
+      <c r="E69" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="70" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B70" t="s">
+        <v>237</v>
+      </c>
+      <c r="C70" t="s">
+        <v>238</v>
+      </c>
+      <c r="D70" t="s">
+        <v>8</v>
+      </c>
+      <c r="E70" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="71" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B71" t="s">
+        <v>192</v>
+      </c>
+      <c r="C71" t="s">
+        <v>241</v>
+      </c>
+      <c r="D71" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="72" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B72" t="s">
+        <v>196</v>
+      </c>
+      <c r="C72" t="s">
+        <v>243</v>
+      </c>
+      <c r="D72" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="73" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B73" t="s">
+        <v>127</v>
+      </c>
+      <c r="C73" t="s">
+        <v>246</v>
+      </c>
+      <c r="D73" t="s">
+        <v>8</v>
+      </c>
+      <c r="E73" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="74" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B74" t="s">
+        <v>153</v>
+      </c>
+      <c r="C74" t="s">
+        <v>249</v>
+      </c>
+      <c r="D74" t="s">
+        <v>8</v>
+      </c>
+      <c r="E74" t="s">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>